<commit_message>
Edits to get the new UCOT reports and fix WBS UCOT report
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WbsBoeReportWithUCOT.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WbsBoeReportWithUCOT.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{482538AE-ED78-4835-A713-D691D9BE0496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F8EC60D-4FEF-4EA2-9F68-605471C2F41E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3030" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WBS Summary of Hours, ODC Costs" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
     <t>Total UCOT Hours</t>
   </si>
   <si>
-    <t>Total Hours with UCOT</t>
+    <t>Grand Total Hours</t>
   </si>
 </sst>
 </file>

</xml_diff>